<commit_message>
Fix formatting issues in a couple validation tables.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/RespiratoryValidation.xlsx
+++ b/data/human/adult/validation/Scenarios/RespiratoryValidation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\dyspnea_update\source\data\human\adult\validation\Scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\release_updates\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{316F1E7B-8667-43E2-846F-5D39022EC7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F378748B-34FC-45FB-88FD-FB12CA044562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8985" yWindow="1935" windowWidth="24135" windowHeight="21030" tabRatio="643" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-2955" windowWidth="29040" windowHeight="15720" tabRatio="643" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="21" r:id="rId1"/>
@@ -4162,7 +4162,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="2" style="1" bestFit="1" customWidth="1"/>
@@ -4255,7 +4255,7 @@
         <v>56</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>99</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">

</xml_diff>